<commit_message>
Login by surname (no password), per-user objects
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CYjpYrVLqaXudpURYJubbc
</commit_message>
<xml_diff>
--- a/google/Шаблон_Заявки_Google.xlsx
+++ b/google/Шаблон_Заявки_Google.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B32"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -565,7 +565,7 @@
     <row r="15" ht="45" customHeight="1">
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>6. Лист «Пользователи»: впишите сотрудников (Email @upiterstroy.ru, ФИО, Роль, Объекты, Активен = Да). Обновите страницу таблицы → меню «Заявки» → «Выдать пароли новым сотрудникам». Каждому на почту уходит письмо со ссылкой, логином и паролем.</t>
+          <t>6. Лист «Пользователи»: впишите сотрудников (Email @upiterstroy.ru, ФИО полностью, Роль, Объекты — код объекта через запятую или «все», Активен = Да). Вход в приложение — по фамилии, без пароля: сотрудник видит только объекты из столбца «Объекты». Однофамильцы входят с инициалами («Иванов И.П.»).</t>
         </is>
       </c>
     </row>
@@ -621,28 +621,28 @@
     <row r="23" ht="24" customHeight="1">
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>Пароли и безопасность</t>
+          <t>Доступ и безопасность</t>
         </is>
       </c>
     </row>
     <row r="24" ht="45" customHeight="1">
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Пароли хранятся только в виде хэша; в письме пароль приходит один раз. Сотрудник может сменить его в приложении (Меню → Сменить пароль). Забыл — выделите его строку на листе «Пользователи» → «Сбросить пароль выбранному сотруднику».</t>
+          <t>Вход по фамилии не защищён паролем: любой, кто знает фамилию сотрудника и ссылку на приложение, увидит его объекты. Данные — заявки и остатки, без платёжной информации. Ссылку на приложение не публикуйте. Каждый вход пишется в лист «Журнал».</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Увольнение: поставьте «Активен = Нет» — вход и синхронизация прекращаются сразу, телефон сможет только работать офлайн с тем, что уже загружено, до следующего подключения.</t>
+          <t>Увольнение: поставьте «Активен = Нет» — вход прекращается сразу; уже вошедший телефон перестаёт синхронизироваться при следующем подключении.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>5 неверных паролей подряд блокируют вход на 15 минут. Вход разрешён только для адресов @upiterstroy.ru.</t>
+          <t>5 неверных попыток с одной и той же фамилией подряд блокируют вход этой фамилии на 15 минут.</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Лимит писем в сутки: до 100 в обычном аккаунте Google и до 1500 в Google Workspace.</t>
+          <t>Письма с паролями больше не отправляются.</t>
         </is>
       </c>
     </row>

</xml_diff>